<commit_message>
Solucionado conexión base de datos
</commit_message>
<xml_diff>
--- a/RPA-EOI/excel/recetas.xlsx
+++ b/RPA-EOI/excel/recetas.xlsx
@@ -25,46 +25,67 @@
     <x:t>Ingrediente</x:t>
   </x:si>
   <x:si>
-    <x:t>3 comensales, 15m, Plato principal, Dificultad baja</x:t>
+    <x:t>nombre</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4 comensales, 45m, Dificultad baja</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>piezas de pollo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Receta de Pollada con arroz</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharadas soperas de ají panca en pasta</x:t>
   </x:si>
   <x:si>
     <x:t>3</x:t>
   </x:si>
   <x:si>
-    <x:t>zucchinis grandes</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
+    <x:t>cucharadas soperas de ajo molido</x:t>
   </x:si>
   <x:si>
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>cebolla chica</x:t>
-  </x:si>
-  <x:si>
-    <x:t>huevos</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cucharada postre de nuez moscada</x:t>
-  </x:si>
-  <x:si>
-    <x:t>½</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cucharada postre de ajo en polvo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>pizca de pimienta</x:t>
-  </x:si>
-  <x:si>
-    <x:t>¼</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cucharada postre de sal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cucharada postre de mostaza</x:t>
+    <x:t>cucharadita de comino molido</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharadita de pimienta negra molida</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharadita de orégano seco molido</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharadas soperas de mostaza</x:t>
+  </x:si>
+  <x:si>
+    <x:t>100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mililitros de vinagre tinto</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mililitros de sillao</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cucharaditas de sal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>aceite c/n</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -415,10 +436,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C9"/>
+  <x:dimension ref="A1:D12"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:3">
+    <x:row r="1" spans="1:4">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -428,93 +449,162 @@
       <x:c r="C1" s="0" t="s">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:3">
+      <x:c r="D1" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:4">
       <x:c r="A2" s="0" t="s">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:4">
       <x:c r="A3" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:3">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:4">
       <x:c r="A4" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>4</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:4">
       <x:c r="A5" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:3">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:4">
       <x:c r="A6" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:4">
+      <x:c r="A7" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:4">
+      <x:c r="A8" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:4">
+      <x:c r="A9" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:4">
+      <x:c r="A10" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:4">
+      <x:c r="A11" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3">
-      <x:c r="A7" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3">
-      <x:c r="A8" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:3">
-      <x:c r="A9" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>16</x:v>
+      <x:c r="C11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:4">
+      <x:c r="A12" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>8</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>